<commit_message>
Add related-articles block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (11):
- blocks/related-articles/related-articles.css
- blocks/related-articles/related-articles.js
- styles/styles.css
- tools/importer/import-article-page.bundle.js
- tools/importer/import-article-page.js
- tools/importer/reports/import-article-page.report.xlsx
- tools/importer/reports/us/en/magazine/arctic-surfing.report.json
- tools/importer/reports/us/en/magazine/guide-la-skateparks.report.json
- tools/importer/reports/us/en/magazine/san-diego-surf.report.json
- tools/importer/reports/us/en/magazine/ski-touring.report.json
- tools/importer/reports/us/en/magazine/western-australia.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-article-page.report.xlsx
+++ b/tools/importer/reports/import-article-page.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="313">
   <si>
     <t>_reportFile</t>
   </si>
@@ -40,7 +40,7 @@
     <t>ca/en.report.json</t>
   </si>
   <si>
-    <t>["carousel-hero","columns","hero","hero","hero","hero","cards","cards"]</t>
+    <t>["carousel-hero","columns","hero","hero","hero","hero","recent-articles","cards"]</t>
   </si>
   <si>
     <t>ca/en</t>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-09-08T20:07:24.167Z</t>
+    <t>2026-09-09T17:26:31.331Z</t>
   </si>
   <si>
     <t>WKND Adventures and Travel</t>
@@ -178,7 +178,7 @@
     <t>us/en</t>
   </si>
   <si>
-    <t>2026-09-08T20:08:09.819Z</t>
+    <t>2026-09-09T17:25:56.576Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en.html</t>
@@ -262,321 +262,324 @@
     <t>ca/en/magazine.report.json</t>
   </si>
   <si>
+    <t>["columns","secure-teasers","secure-teasers","cards"]</t>
+  </si>
+  <si>
+    <t>ca/en/magazine</t>
+  </si>
+  <si>
+    <t>2026-09-09T19:14:25.327Z</t>
+  </si>
+  <si>
+    <t>Magazine</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/magazine.html</t>
+  </si>
+  <si>
+    <t>us/en/about-us.report.json</t>
+  </si>
+  <si>
+    <t>us/en/about-us</t>
+  </si>
+  <si>
+    <t>2026-09-08T20:47:50.809Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/about-us.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures</t>
+  </si>
+  <si>
+    <t>2026-09-08T20:59:25.298Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures.html</t>
+  </si>
+  <si>
+    <t>us/en/faqs.report.json</t>
+  </si>
+  <si>
+    <t>us/en/faqs</t>
+  </si>
+  <si>
+    <t>2026-09-08T21:08:28.532Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/faqs.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine</t>
+  </si>
+  <si>
+    <t>2026-09-09T19:14:21.177Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/bali-surf-camp.report.json</t>
+  </si>
+  <si>
+    <t>["carousel-gallery","table-specs","table-specs","table-specs","table-specs","table-specs","table-specs","table-specs","table-specs","tabs-detail","tabs-detail"]</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/bali-surf-camp</t>
+  </si>
+  <si>
+    <t>adventure-detail</t>
+  </si>
+  <si>
+    <t>2026-09-08T18:50:23.840Z</t>
+  </si>
+  <si>
+    <t>Bali Surf Camp</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/bali-surf-camp.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/beervana-portland.report.json</t>
+  </si>
+  <si>
+    <t>["carousel-gallery","table-specs","table-specs","table-specs","table-specs","tabs-detail","tabs-detail"]</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/beervana-portland</t>
+  </si>
+  <si>
+    <t>2026-09-08T18:50:29.661Z</t>
+  </si>
+  <si>
+    <t>Beervana in Portland</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/beervana-portland.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/climbing-new-zealand.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/climbing-new-zealand</t>
+  </si>
+  <si>
+    <t>2026-09-08T18:50:34.351Z</t>
+  </si>
+  <si>
+    <t>Climbing New Zealand</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/climbing-new-zealand.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/colorado-rock-climbing.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/colorado-rock-climbing</t>
+  </si>
+  <si>
+    <t>2026-09-08T18:50:38.993Z</t>
+  </si>
+  <si>
+    <t>Colorado Rock Climbing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/colorado-rock-climbing.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/cycling-southern-utah.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/cycling-southern-utah</t>
+  </si>
+  <si>
+    <t>2026-09-08T18:50:43.820Z</t>
+  </si>
+  <si>
+    <t>Cycling Southern Utah</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/cycling-southern-utah.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/cycling-tuscany.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/cycling-tuscany</t>
+  </si>
+  <si>
+    <t>2026-09-08T18:50:48.795Z</t>
+  </si>
+  <si>
+    <t>Cycling Tuscany</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/cycling-tuscany.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/downhill-skiing-wyoming.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/downhill-skiing-wyoming</t>
+  </si>
+  <si>
+    <t>2026-09-08T18:50:54.144Z</t>
+  </si>
+  <si>
+    <t>Downhill Skiing Wyoming</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/downhill-skiing-wyoming.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/gastronomic-marais-tour.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/gastronomic-marais-tour</t>
+  </si>
+  <si>
+    <t>2026-09-08T18:51:00.912Z</t>
+  </si>
+  <si>
+    <t>Gastronomic Marais Tour</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/gastronomic-marais-tour.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/napa-wine-tasting.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/napa-wine-tasting</t>
+  </si>
+  <si>
+    <t>2026-09-08T18:51:05.164Z</t>
+  </si>
+  <si>
+    <t>Napa Wine Tasting</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/napa-wine-tasting.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/riverside-camping-australia.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/riverside-camping-australia</t>
+  </si>
+  <si>
+    <t>2026-09-08T18:51:10.701Z</t>
+  </si>
+  <si>
+    <t>Riverside Camping</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/riverside-camping-australia.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/ski-touring-mont-blanc.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/ski-touring-mont-blanc</t>
+  </si>
+  <si>
+    <t>2026-09-08T18:51:16.120Z</t>
+  </si>
+  <si>
+    <t>Ski Touring Mont Blanc</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/ski-touring-mont-blanc.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/surf-camp-costa-rica.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/surf-camp-costa-rica</t>
+  </si>
+  <si>
+    <t>2026-09-08T18:51:21.295Z</t>
+  </si>
+  <si>
+    <t>Surf Camp in Costa Rica</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/surf-camp-costa-rica.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/tahoe-skiing.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/tahoe-skiing</t>
+  </si>
+  <si>
+    <t>2026-09-08T18:51:25.230Z</t>
+  </si>
+  <si>
+    <t>Tahoe Skiing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/tahoe-skiing.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/west-coast-cycling.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/west-coast-cycling</t>
+  </si>
+  <si>
+    <t>2026-09-08T18:51:30.182Z</t>
+  </si>
+  <si>
+    <t>West Coast Cycling</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/west-coast-cycling.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/whistler-mountain-biking.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/whistler-mountain-biking</t>
+  </si>
+  <si>
+    <t>2026-09-08T18:51:35.795Z</t>
+  </si>
+  <si>
+    <t>Whistler Mountain Biking</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/whistler-mountain-biking.html</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/yosemite-backpacking.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/adventures/yosemite-backpacking</t>
+  </si>
+  <si>
+    <t>2026-09-08T18:51:40.693Z</t>
+  </si>
+  <si>
+    <t>Yosemite Backpacking</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/adventures/yosemite-backpacking.html</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/arctic-surfing.report.json</t>
+  </si>
+  <si>
     <t>[]</t>
   </si>
   <si>
-    <t>ca/en/magazine</t>
-  </si>
-  <si>
-    <t>2026-09-08T20:47:39.369Z</t>
-  </si>
-  <si>
-    <t>Magazine</t>
-  </si>
-  <si>
-    <t>https://wknd.site/ca/en/magazine.html</t>
-  </si>
-  <si>
-    <t>us/en/about-us.report.json</t>
-  </si>
-  <si>
-    <t>us/en/about-us</t>
-  </si>
-  <si>
-    <t>2026-09-08T20:47:50.809Z</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/about-us.html</t>
-  </si>
-  <si>
-    <t>us/en/adventures.report.json</t>
-  </si>
-  <si>
-    <t>us/en/adventures</t>
-  </si>
-  <si>
-    <t>2026-09-08T20:59:25.298Z</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/adventures.html</t>
-  </si>
-  <si>
-    <t>us/en/faqs.report.json</t>
-  </si>
-  <si>
-    <t>us/en/faqs</t>
-  </si>
-  <si>
-    <t>2026-09-08T21:08:28.532Z</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/faqs.html</t>
-  </si>
-  <si>
-    <t>us/en/magazine.report.json</t>
-  </si>
-  <si>
-    <t>us/en/magazine</t>
-  </si>
-  <si>
-    <t>2026-09-08T20:47:56.405Z</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/magazine.html</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/bali-surf-camp.report.json</t>
-  </si>
-  <si>
-    <t>["carousel-gallery","table-specs","table-specs","table-specs","table-specs","table-specs","table-specs","table-specs","table-specs","tabs-detail","tabs-detail"]</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/bali-surf-camp</t>
-  </si>
-  <si>
-    <t>adventure-detail</t>
-  </si>
-  <si>
-    <t>2026-09-08T18:50:23.840Z</t>
-  </si>
-  <si>
-    <t>Bali Surf Camp</t>
-  </si>
-  <si>
-    <t>https://wknd.site/ca/en/adventures/bali-surf-camp.html</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/beervana-portland.report.json</t>
-  </si>
-  <si>
-    <t>["carousel-gallery","table-specs","table-specs","table-specs","table-specs","tabs-detail","tabs-detail"]</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/beervana-portland</t>
-  </si>
-  <si>
-    <t>2026-09-08T18:50:29.661Z</t>
-  </si>
-  <si>
-    <t>Beervana in Portland</t>
-  </si>
-  <si>
-    <t>https://wknd.site/ca/en/adventures/beervana-portland.html</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/climbing-new-zealand.report.json</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/climbing-new-zealand</t>
-  </si>
-  <si>
-    <t>2026-09-08T18:50:34.351Z</t>
-  </si>
-  <si>
-    <t>Climbing New Zealand</t>
-  </si>
-  <si>
-    <t>https://wknd.site/ca/en/adventures/climbing-new-zealand.html</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/colorado-rock-climbing.report.json</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/colorado-rock-climbing</t>
-  </si>
-  <si>
-    <t>2026-09-08T18:50:38.993Z</t>
-  </si>
-  <si>
-    <t>Colorado Rock Climbing</t>
-  </si>
-  <si>
-    <t>https://wknd.site/ca/en/adventures/colorado-rock-climbing.html</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/cycling-southern-utah.report.json</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/cycling-southern-utah</t>
-  </si>
-  <si>
-    <t>2026-09-08T18:50:43.820Z</t>
-  </si>
-  <si>
-    <t>Cycling Southern Utah</t>
-  </si>
-  <si>
-    <t>https://wknd.site/ca/en/adventures/cycling-southern-utah.html</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/cycling-tuscany.report.json</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/cycling-tuscany</t>
-  </si>
-  <si>
-    <t>2026-09-08T18:50:48.795Z</t>
-  </si>
-  <si>
-    <t>Cycling Tuscany</t>
-  </si>
-  <si>
-    <t>https://wknd.site/ca/en/adventures/cycling-tuscany.html</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/downhill-skiing-wyoming.report.json</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/downhill-skiing-wyoming</t>
-  </si>
-  <si>
-    <t>2026-09-08T18:50:54.144Z</t>
-  </si>
-  <si>
-    <t>Downhill Skiing Wyoming</t>
-  </si>
-  <si>
-    <t>https://wknd.site/ca/en/adventures/downhill-skiing-wyoming.html</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/gastronomic-marais-tour.report.json</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/gastronomic-marais-tour</t>
-  </si>
-  <si>
-    <t>2026-09-08T18:51:00.912Z</t>
-  </si>
-  <si>
-    <t>Gastronomic Marais Tour</t>
-  </si>
-  <si>
-    <t>https://wknd.site/ca/en/adventures/gastronomic-marais-tour.html</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/napa-wine-tasting.report.json</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/napa-wine-tasting</t>
-  </si>
-  <si>
-    <t>2026-09-08T18:51:05.164Z</t>
-  </si>
-  <si>
-    <t>Napa Wine Tasting</t>
-  </si>
-  <si>
-    <t>https://wknd.site/ca/en/adventures/napa-wine-tasting.html</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/riverside-camping-australia.report.json</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/riverside-camping-australia</t>
-  </si>
-  <si>
-    <t>2026-09-08T18:51:10.701Z</t>
-  </si>
-  <si>
-    <t>Riverside Camping</t>
-  </si>
-  <si>
-    <t>https://wknd.site/ca/en/adventures/riverside-camping-australia.html</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/ski-touring-mont-blanc.report.json</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/ski-touring-mont-blanc</t>
-  </si>
-  <si>
-    <t>2026-09-08T18:51:16.120Z</t>
-  </si>
-  <si>
-    <t>Ski Touring Mont Blanc</t>
-  </si>
-  <si>
-    <t>https://wknd.site/ca/en/adventures/ski-touring-mont-blanc.html</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/surf-camp-costa-rica.report.json</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/surf-camp-costa-rica</t>
-  </si>
-  <si>
-    <t>2026-09-08T18:51:21.295Z</t>
-  </si>
-  <si>
-    <t>Surf Camp in Costa Rica</t>
-  </si>
-  <si>
-    <t>https://wknd.site/ca/en/adventures/surf-camp-costa-rica.html</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/tahoe-skiing.report.json</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/tahoe-skiing</t>
-  </si>
-  <si>
-    <t>2026-09-08T18:51:25.230Z</t>
-  </si>
-  <si>
-    <t>Tahoe Skiing</t>
-  </si>
-  <si>
-    <t>https://wknd.site/ca/en/adventures/tahoe-skiing.html</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/west-coast-cycling.report.json</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/west-coast-cycling</t>
-  </si>
-  <si>
-    <t>2026-09-08T18:51:30.182Z</t>
-  </si>
-  <si>
-    <t>West Coast Cycling</t>
-  </si>
-  <si>
-    <t>https://wknd.site/ca/en/adventures/west-coast-cycling.html</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/whistler-mountain-biking.report.json</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/whistler-mountain-biking</t>
-  </si>
-  <si>
-    <t>2026-09-08T18:51:35.795Z</t>
-  </si>
-  <si>
-    <t>Whistler Mountain Biking</t>
-  </si>
-  <si>
-    <t>https://wknd.site/ca/en/adventures/whistler-mountain-biking.html</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/yosemite-backpacking.report.json</t>
-  </si>
-  <si>
-    <t>ca/en/adventures/yosemite-backpacking</t>
-  </si>
-  <si>
-    <t>2026-09-08T18:51:40.693Z</t>
-  </si>
-  <si>
-    <t>Yosemite Backpacking</t>
-  </si>
-  <si>
-    <t>https://wknd.site/ca/en/adventures/yosemite-backpacking.html</t>
-  </si>
-  <si>
-    <t>ca/en/magazine/arctic-surfing.report.json</t>
-  </si>
-  <si>
     <t>ca/en/magazine/arctic-surfing</t>
   </si>
   <si>
@@ -865,7 +868,7 @@
     <t>us/en/magazine/arctic-surfing</t>
   </si>
   <si>
-    <t>2026-09-09T16:53:54.843Z</t>
+    <t>2026-09-09T19:51:32.413Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/magazine/arctic-surfing.html</t>
@@ -877,7 +880,7 @@
     <t>us/en/magazine/guide-la-skateparks</t>
   </si>
   <si>
-    <t>2026-09-09T16:53:59.991Z</t>
+    <t>2026-09-09T19:51:36.344Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/magazine/guide-la-skateparks.html</t>
@@ -889,7 +892,7 @@
     <t>us/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-09-09T16:54:04.869Z</t>
+    <t>2026-09-09T19:51:42.282Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/magazine/san-diego-surf.html</t>
@@ -901,7 +904,7 @@
     <t>us/en/magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-09-09T16:54:10.205Z</t>
+    <t>2026-09-09T19:51:46.067Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/magazine/ski-touring.html</t>
@@ -913,7 +916,7 @@
     <t>us/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-09-09T16:54:15.560Z</t>
+    <t>2026-09-09T19:51:50.555Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/magazine/western-australia.html</t>
@@ -2286,62 +2289,62 @@
         <v>187</v>
       </c>
       <c r="B37" t="s">
-        <v>83</v>
+        <v>188</v>
       </c>
       <c r="C37" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D37" t="s">
         <v>11</v>
       </c>
       <c r="E37" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F37" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G37" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H37" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B38" t="s">
-        <v>83</v>
+        <v>188</v>
       </c>
       <c r="C38" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D38" t="s">
         <v>11</v>
       </c>
       <c r="E38" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F38" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G38" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H38" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B39" t="s">
-        <v>83</v>
+        <v>188</v>
       </c>
       <c r="C39" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D39" t="s">
         <v>11</v>
@@ -2350,102 +2353,102 @@
         <v>64</v>
       </c>
       <c r="F39" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G39" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H39" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B40" t="s">
-        <v>83</v>
+        <v>188</v>
       </c>
       <c r="C40" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D40" t="s">
         <v>11</v>
       </c>
       <c r="E40" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F40" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="G40" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H40" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B41" t="s">
-        <v>83</v>
+        <v>188</v>
       </c>
       <c r="C41" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D41" t="s">
         <v>11</v>
       </c>
       <c r="E41" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F41" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G41" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H41" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B42" t="s">
-        <v>83</v>
+        <v>188</v>
       </c>
       <c r="C42" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D42" t="s">
         <v>11</v>
       </c>
       <c r="E42" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F42" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="G42" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="H42" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B43" t="s">
         <v>105</v>
       </c>
       <c r="C43" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D43" t="s">
         <v>11</v>
@@ -2454,24 +2457,24 @@
         <v>107</v>
       </c>
       <c r="F43" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G43" t="s">
         <v>109</v>
       </c>
       <c r="H43" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B44" t="s">
         <v>112</v>
       </c>
       <c r="C44" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D44" t="s">
         <v>11</v>
@@ -2480,24 +2483,24 @@
         <v>107</v>
       </c>
       <c r="F44" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="G44" t="s">
         <v>115</v>
       </c>
       <c r="H44" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B45" t="s">
         <v>112</v>
       </c>
       <c r="C45" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D45" t="s">
         <v>11</v>
@@ -2506,24 +2509,24 @@
         <v>107</v>
       </c>
       <c r="F45" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G45" t="s">
         <v>120</v>
       </c>
       <c r="H45" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B46" t="s">
         <v>112</v>
       </c>
       <c r="C46" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D46" t="s">
         <v>11</v>
@@ -2532,24 +2535,24 @@
         <v>107</v>
       </c>
       <c r="F46" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="G46" t="s">
         <v>125</v>
       </c>
       <c r="H46" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B47" t="s">
         <v>112</v>
       </c>
       <c r="C47" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D47" t="s">
         <v>11</v>
@@ -2558,24 +2561,24 @@
         <v>107</v>
       </c>
       <c r="F47" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="G47" t="s">
         <v>130</v>
       </c>
       <c r="H47" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B48" t="s">
         <v>112</v>
       </c>
       <c r="C48" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D48" t="s">
         <v>11</v>
@@ -2584,24 +2587,24 @@
         <v>107</v>
       </c>
       <c r="F48" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="G48" t="s">
         <v>135</v>
       </c>
       <c r="H48" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B49" t="s">
         <v>112</v>
       </c>
       <c r="C49" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D49" t="s">
         <v>11</v>
@@ -2610,24 +2613,24 @@
         <v>107</v>
       </c>
       <c r="F49" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="G49" t="s">
         <v>140</v>
       </c>
       <c r="H49" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B50" t="s">
         <v>112</v>
       </c>
       <c r="C50" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D50" t="s">
         <v>11</v>
@@ -2636,24 +2639,24 @@
         <v>107</v>
       </c>
       <c r="F50" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G50" t="s">
         <v>145</v>
       </c>
       <c r="H50" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B51" t="s">
         <v>112</v>
       </c>
       <c r="C51" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D51" t="s">
         <v>11</v>
@@ -2662,24 +2665,24 @@
         <v>107</v>
       </c>
       <c r="F51" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="G51" t="s">
         <v>150</v>
       </c>
       <c r="H51" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B52" t="s">
         <v>112</v>
       </c>
       <c r="C52" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D52" t="s">
         <v>11</v>
@@ -2688,24 +2691,24 @@
         <v>107</v>
       </c>
       <c r="F52" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G52" t="s">
         <v>155</v>
       </c>
       <c r="H52" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B53" t="s">
         <v>112</v>
       </c>
       <c r="C53" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D53" t="s">
         <v>11</v>
@@ -2714,24 +2717,24 @@
         <v>107</v>
       </c>
       <c r="F53" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="G53" t="s">
         <v>160</v>
       </c>
       <c r="H53" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B54" t="s">
         <v>112</v>
       </c>
       <c r="C54" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D54" t="s">
         <v>11</v>
@@ -2740,24 +2743,24 @@
         <v>107</v>
       </c>
       <c r="F54" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="G54" t="s">
         <v>165</v>
       </c>
       <c r="H54" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B55" t="s">
         <v>112</v>
       </c>
       <c r="C55" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D55" t="s">
         <v>11</v>
@@ -2766,24 +2769,24 @@
         <v>107</v>
       </c>
       <c r="F55" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="G55" t="s">
         <v>170</v>
       </c>
       <c r="H55" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B56" t="s">
         <v>112</v>
       </c>
       <c r="C56" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D56" t="s">
         <v>11</v>
@@ -2792,24 +2795,24 @@
         <v>107</v>
       </c>
       <c r="F56" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="G56" t="s">
         <v>175</v>
       </c>
       <c r="H56" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B57" t="s">
         <v>112</v>
       </c>
       <c r="C57" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D57" t="s">
         <v>11</v>
@@ -2818,24 +2821,24 @@
         <v>107</v>
       </c>
       <c r="F57" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="G57" t="s">
         <v>180</v>
       </c>
       <c r="H57" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B58" t="s">
         <v>112</v>
       </c>
       <c r="C58" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D58" t="s">
         <v>11</v>
@@ -2844,195 +2847,195 @@
         <v>107</v>
       </c>
       <c r="F58" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G58" t="s">
         <v>185</v>
       </c>
       <c r="H58" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B59" t="s">
-        <v>83</v>
+        <v>188</v>
       </c>
       <c r="C59" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D59" t="s">
         <v>11</v>
       </c>
       <c r="E59" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F59" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="G59" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="H59" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B60" t="s">
-        <v>83</v>
+        <v>188</v>
       </c>
       <c r="C60" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D60" t="s">
         <v>11</v>
       </c>
       <c r="E60" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F60" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="G60" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="H60" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B61" t="s">
-        <v>83</v>
+        <v>188</v>
       </c>
       <c r="C61" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D61" t="s">
         <v>11</v>
       </c>
       <c r="E61" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F61" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="G61" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H61" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B62" t="s">
-        <v>83</v>
+        <v>188</v>
       </c>
       <c r="C62" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D62" t="s">
         <v>11</v>
       </c>
       <c r="E62" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F62" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="G62" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H62" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B63" t="s">
-        <v>83</v>
+        <v>188</v>
       </c>
       <c r="C63" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D63" t="s">
         <v>11</v>
       </c>
       <c r="E63" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F63" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="G63" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="H63" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B64" t="s">
-        <v>83</v>
+        <v>188</v>
       </c>
       <c r="C64" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D64" t="s">
         <v>11</v>
       </c>
       <c r="E64" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F64" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="G64" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="H64" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B65" t="s">
-        <v>83</v>
+        <v>188</v>
       </c>
       <c r="C65" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D65" t="s">
         <v>11</v>
       </c>
       <c r="E65" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F65" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="G65" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="H65" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
   </sheetData>

</xml_diff>